<commit_message>
Fixed all test cases
</commit_message>
<xml_diff>
--- a/src/data/Auction_Units.xlsx
+++ b/src/data/Auction_Units.xlsx
@@ -691,16 +691,16 @@
         <v>221121</v>
       </c>
       <c r="AT2" t="str">
-        <v>06-09-2026</v>
+        <v>11-09-2026</v>
       </c>
       <c r="AU2" t="str">
-        <v>14:57</v>
+        <v>17:42</v>
       </c>
       <c r="AV2" t="str">
-        <v>06-09-2026</v>
+        <v>11-09-2026</v>
       </c>
       <c r="AW2" t="str">
-        <v>16:57</v>
+        <v>17:46</v>
       </c>
       <c r="AX2">
         <v>900</v>

</xml_diff>

<commit_message>
Checked and working suits
</commit_message>
<xml_diff>
--- a/src/data/Auction_Units.xlsx
+++ b/src/data/Auction_Units.xlsx
@@ -691,16 +691,16 @@
         <v>221121</v>
       </c>
       <c r="AT2" t="str">
-        <v>11-09-2026</v>
+        <v>21-09-2026</v>
       </c>
       <c r="AU2" t="str">
-        <v>17:42</v>
+        <v>17:50</v>
       </c>
       <c r="AV2" t="str">
-        <v>11-09-2026</v>
+        <v>21-09-2026</v>
       </c>
       <c r="AW2" t="str">
-        <v>17:46</v>
+        <v>17:54</v>
       </c>
       <c r="AX2">
         <v>900</v>

</xml_diff>

<commit_message>
added steps to all test cases except e2e
</commit_message>
<xml_diff>
--- a/src/data/Auction_Units.xlsx
+++ b/src/data/Auction_Units.xlsx
@@ -691,16 +691,16 @@
         <v>221121</v>
       </c>
       <c r="AT2" t="str">
-        <v>21-09-2026</v>
+        <v>22-09-2026</v>
       </c>
       <c r="AU2" t="str">
-        <v>17:50</v>
+        <v>11:41</v>
       </c>
       <c r="AV2" t="str">
-        <v>21-09-2026</v>
+        <v>22-09-2026</v>
       </c>
       <c r="AW2" t="str">
-        <v>17:54</v>
+        <v>11:45</v>
       </c>
       <c r="AX2">
         <v>900</v>

</xml_diff>